<commit_message>
weather data and image trajectories updated with new data. Flight1 left out of hlangwine!
</commit_message>
<xml_diff>
--- a/data/in/Additonal Weather data A Davies.xlsx
+++ b/data/in/Additonal Weather data A Davies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0d208f1c5c7e8ef3/Documents/Python/ThermalLandscapes/data/in/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{61AFDC31-8994-4967-ACB7-007959086D55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BF05CA9-D5B9-414E-9793-5A3047923DA2}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{61AFDC31-8994-4967-ACB7-007959086D55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1ACE9A0-C955-46DE-97E7-CC0EAF8F2E00}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="75" yWindow="6405" windowWidth="29100" windowHeight="13995" activeTab="1" xr2:uid="{4F82AF74-0B02-4487-A9FC-0C348CF57722}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4F82AF74-0B02-4487-A9FC-0C348CF57722}"/>
   </bookViews>
   <sheets>
     <sheet name="shingwedzi" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="87">
   <si>
     <t>4 Dec 01:00</t>
   </si>
@@ -359,6 +359,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -658,30 +662,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3010B0C4-60EE-4EA2-9945-4BDD3DEFF21F}">
-  <dimension ref="A1:AC25"/>
+  <dimension ref="A1:Z49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>36</v>
-      </c>
-      <c r="F1" t="s">
-        <v>37</v>
       </c>
       <c r="G1" t="s">
         <v>37</v>
@@ -731,49 +735,28 @@
       <c r="V1" t="s">
         <v>52</v>
       </c>
-      <c r="W1" t="s">
-        <v>53</v>
-      </c>
-      <c r="X1" t="s">
-        <v>54</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>55</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>56</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>57</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>58</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
+    </row>
+    <row r="2" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1">
         <v>44169</v>
       </c>
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2">
+      <c r="C2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="2">
         <v>22.39</v>
       </c>
-      <c r="D2" s="2">
+      <c r="E2" s="2">
         <v>22.62</v>
       </c>
-      <c r="E2" s="2">
+      <c r="F2" s="2">
         <v>22.29</v>
       </c>
-      <c r="F2" s="2">
+      <c r="G2" s="2">
         <v>66.5</v>
-      </c>
-      <c r="G2" s="2">
-        <v>0</v>
       </c>
       <c r="H2" s="2">
         <v>15.85</v>
@@ -820,49 +803,32 @@
       <c r="V2" t="s">
         <v>2</v>
       </c>
-      <c r="W2" s="2">
-        <v>0</v>
-      </c>
-      <c r="X2" s="2">
-        <v>18.16</v>
-      </c>
-      <c r="Y2" t="s">
+      <c r="W2" s="2"/>
+      <c r="X2" s="2"/>
+      <c r="Y2" s="2"/>
+      <c r="Z2" s="2"/>
+    </row>
+    <row r="3" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="Z2" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+      <c r="B3" s="1">
         <v>44169</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="2">
+      <c r="D3" s="2">
         <v>22.49</v>
       </c>
-      <c r="D3" s="2">
+      <c r="E3" s="2">
         <v>22.68</v>
       </c>
-      <c r="E3" s="2">
+      <c r="F3" s="2">
         <v>22.37</v>
       </c>
-      <c r="F3" s="2">
+      <c r="G3" s="2">
         <v>66</v>
-      </c>
-      <c r="G3" s="2">
-        <v>0</v>
       </c>
       <c r="H3" s="2">
         <v>15.82</v>
@@ -909,49 +875,32 @@
       <c r="V3" t="s">
         <v>2</v>
       </c>
-      <c r="W3" s="2">
-        <v>0</v>
-      </c>
-      <c r="X3" s="2">
-        <v>18.18</v>
-      </c>
-      <c r="Y3" t="s">
+      <c r="W3" s="2"/>
+      <c r="X3" s="2"/>
+      <c r="Y3" s="2"/>
+      <c r="Z3" s="2"/>
+    </row>
+    <row r="4" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="Z3" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC3" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
+      <c r="B4" s="1">
         <v>44169</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="2">
+      <c r="D4" s="2">
         <v>22.67</v>
       </c>
-      <c r="D4" s="2">
+      <c r="E4" s="2">
         <v>22.79</v>
       </c>
-      <c r="E4" s="2">
+      <c r="F4" s="2">
         <v>22.46</v>
       </c>
-      <c r="F4" s="2">
+      <c r="G4" s="2">
         <v>66.3</v>
-      </c>
-      <c r="G4" s="2">
-        <v>0</v>
       </c>
       <c r="H4" s="2">
         <v>16.059999999999999</v>
@@ -998,49 +947,32 @@
       <c r="V4" t="s">
         <v>2</v>
       </c>
-      <c r="W4" s="2">
-        <v>0</v>
-      </c>
-      <c r="X4" s="2">
-        <v>18.38</v>
-      </c>
-      <c r="Y4" t="s">
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="2"/>
+      <c r="Z4" s="2"/>
+    </row>
+    <row r="5" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="Z4" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA4" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB4" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
+      <c r="B5" s="1">
         <v>44169</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="2">
+      <c r="D5" s="2">
         <v>21.77</v>
       </c>
-      <c r="D5" s="2">
+      <c r="E5" s="2">
         <v>22.36</v>
       </c>
-      <c r="E5" s="2">
+      <c r="F5" s="2">
         <v>21.41</v>
       </c>
-      <c r="F5" s="2">
+      <c r="G5" s="2">
         <v>68.900000000000006</v>
-      </c>
-      <c r="G5" s="2">
-        <v>0</v>
       </c>
       <c r="H5" s="2">
         <v>15.81</v>
@@ -1087,49 +1019,32 @@
       <c r="V5" t="s">
         <v>2</v>
       </c>
-      <c r="W5" s="2">
-        <v>0</v>
-      </c>
-      <c r="X5" s="2">
-        <v>17.920000000000002</v>
-      </c>
-      <c r="Y5" t="s">
+      <c r="W5" s="2"/>
+      <c r="X5" s="2"/>
+      <c r="Y5" s="2"/>
+      <c r="Z5" s="2"/>
+    </row>
+    <row r="6" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>3</v>
       </c>
-      <c r="Z5" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC5" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
+      <c r="B6" s="1">
         <v>44169</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="2">
+      <c r="D6" s="2">
         <v>21.07</v>
       </c>
-      <c r="D6" s="2">
+      <c r="E6" s="2">
         <v>21.3</v>
       </c>
-      <c r="E6" s="2">
+      <c r="F6" s="2">
         <v>21.04</v>
       </c>
-      <c r="F6" s="2">
+      <c r="G6" s="2">
         <v>70.7</v>
-      </c>
-      <c r="G6" s="2">
-        <v>0</v>
       </c>
       <c r="H6" s="2">
         <v>15.54</v>
@@ -1176,49 +1091,32 @@
       <c r="V6" t="s">
         <v>2</v>
       </c>
-      <c r="W6" s="2">
-        <v>0</v>
-      </c>
-      <c r="X6" s="2">
-        <v>17.53</v>
-      </c>
-      <c r="Y6" t="s">
+      <c r="W6" s="2"/>
+      <c r="X6" s="2"/>
+      <c r="Y6" s="2"/>
+      <c r="Z6" s="2"/>
+    </row>
+    <row r="7" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="Z6" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA6" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB6" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC6" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
+      <c r="B7" s="1">
         <v>44169</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="2">
+      <c r="D7" s="2">
         <v>21.64</v>
       </c>
-      <c r="D7" s="2">
+      <c r="E7" s="2">
         <v>22.46</v>
       </c>
-      <c r="E7" s="2">
+      <c r="F7" s="2">
         <v>21.07</v>
       </c>
-      <c r="F7" s="2">
+      <c r="G7" s="2">
         <v>70.2</v>
-      </c>
-      <c r="G7" s="2">
-        <v>0</v>
       </c>
       <c r="H7" s="2">
         <v>15.98</v>
@@ -1265,49 +1163,32 @@
       <c r="V7" t="s">
         <v>2</v>
       </c>
-      <c r="W7" s="2">
-        <v>0</v>
-      </c>
-      <c r="X7" s="2">
-        <v>17.98</v>
-      </c>
-      <c r="Y7" t="s">
+      <c r="W7" s="2"/>
+      <c r="X7" s="2"/>
+      <c r="Y7" s="2"/>
+      <c r="Z7" s="2"/>
+    </row>
+    <row r="8" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>3</v>
       </c>
-      <c r="Z7" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA7" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB7" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC7" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
+      <c r="B8" s="1">
         <v>44169</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="2">
+      <c r="D8" s="2">
         <v>23.91</v>
       </c>
-      <c r="D8" s="2">
+      <c r="E8" s="2">
         <v>24.35</v>
       </c>
-      <c r="E8" s="2">
+      <c r="F8" s="2">
         <v>22.81</v>
       </c>
-      <c r="F8" s="2">
+      <c r="G8" s="2">
         <v>68.3</v>
-      </c>
-      <c r="G8" s="2">
-        <v>0</v>
       </c>
       <c r="H8" s="2">
         <v>17.71</v>
@@ -1354,49 +1235,32 @@
       <c r="V8" t="s">
         <v>2</v>
       </c>
-      <c r="W8" s="2">
-        <v>0</v>
-      </c>
-      <c r="X8" s="2">
-        <v>19.77</v>
-      </c>
-      <c r="Y8" t="s">
+      <c r="W8" s="2"/>
+      <c r="X8" s="2"/>
+      <c r="Y8" s="2"/>
+      <c r="Z8" s="2"/>
+    </row>
+    <row r="9" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>3</v>
       </c>
-      <c r="Z8" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA8" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB8" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC8" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
+      <c r="B9" s="1">
         <v>44169</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="2">
+      <c r="D9" s="2">
         <v>25.12</v>
       </c>
-      <c r="D9" s="2">
+      <c r="E9" s="2">
         <v>25.82</v>
       </c>
-      <c r="E9" s="2">
+      <c r="F9" s="2">
         <v>24.38</v>
       </c>
-      <c r="F9" s="2">
+      <c r="G9" s="2">
         <v>67.8</v>
-      </c>
-      <c r="G9" s="2">
-        <v>0</v>
       </c>
       <c r="H9" s="2">
         <v>18.75</v>
@@ -1443,49 +1307,32 @@
       <c r="V9" t="s">
         <v>2</v>
       </c>
-      <c r="W9" s="2">
-        <v>0</v>
-      </c>
-      <c r="X9" s="2">
-        <v>20.79</v>
-      </c>
-      <c r="Y9" t="s">
+      <c r="W9" s="2"/>
+      <c r="X9" s="2"/>
+      <c r="Y9" s="2"/>
+      <c r="Z9" s="2"/>
+    </row>
+    <row r="10" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>3</v>
       </c>
-      <c r="Z9" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA9" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB9" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC9" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
+      <c r="B10" s="1">
         <v>44169</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="2">
+      <c r="D10" s="2">
         <v>28.6</v>
       </c>
-      <c r="D10" s="2">
+      <c r="E10" s="2">
         <v>29.79</v>
       </c>
-      <c r="E10" s="2">
+      <c r="F10" s="2">
         <v>26.22</v>
       </c>
-      <c r="F10" s="2">
+      <c r="G10" s="2">
         <v>60.3</v>
-      </c>
-      <c r="G10" s="2">
-        <v>0</v>
       </c>
       <c r="H10" s="2">
         <v>20.149999999999999</v>
@@ -1532,49 +1379,32 @@
       <c r="V10" t="s">
         <v>2</v>
       </c>
-      <c r="W10" s="2">
-        <v>0</v>
-      </c>
-      <c r="X10" s="2">
-        <v>22.71</v>
-      </c>
-      <c r="Y10" t="s">
+      <c r="W10" s="2"/>
+      <c r="X10" s="2"/>
+      <c r="Y10" s="2"/>
+      <c r="Z10" s="2"/>
+    </row>
+    <row r="11" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>3</v>
       </c>
-      <c r="Z10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC10" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
+      <c r="B11" s="1">
         <v>44169</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="2">
+      <c r="D11" s="2">
         <v>30.86</v>
       </c>
-      <c r="D11" s="2">
+      <c r="E11" s="2">
         <v>31.59</v>
       </c>
-      <c r="E11" s="2">
+      <c r="F11" s="2">
         <v>29.84</v>
       </c>
-      <c r="F11" s="2">
+      <c r="G11" s="2">
         <v>52.9</v>
-      </c>
-      <c r="G11" s="2">
-        <v>0</v>
       </c>
       <c r="H11" s="2">
         <v>20.13</v>
@@ -1621,49 +1451,32 @@
       <c r="V11" t="s">
         <v>2</v>
       </c>
-      <c r="W11" s="2">
-        <v>0</v>
-      </c>
-      <c r="X11" s="2">
-        <v>23.34</v>
-      </c>
-      <c r="Y11" t="s">
+      <c r="W11" s="2"/>
+      <c r="X11" s="2"/>
+      <c r="Y11" s="2"/>
+      <c r="Z11" s="2"/>
+    </row>
+    <row r="12" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>3</v>
       </c>
-      <c r="Z11" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA11" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB11" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC11" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
+      <c r="B12" s="1">
         <v>44169</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="2">
+      <c r="D12" s="2">
         <v>31.34</v>
       </c>
-      <c r="D12" s="2">
+      <c r="E12" s="2">
         <v>31.98</v>
       </c>
-      <c r="E12" s="2">
+      <c r="F12" s="2">
         <v>30.9</v>
       </c>
-      <c r="F12" s="2">
+      <c r="G12" s="2">
         <v>51.2</v>
-      </c>
-      <c r="G12" s="2">
-        <v>0</v>
       </c>
       <c r="H12" s="2">
         <v>20.05</v>
@@ -1710,49 +1523,32 @@
       <c r="V12" t="s">
         <v>2</v>
       </c>
-      <c r="W12" s="2">
-        <v>0</v>
-      </c>
-      <c r="X12" s="2">
-        <v>23.43</v>
-      </c>
-      <c r="Y12" t="s">
+      <c r="W12" s="2"/>
+      <c r="X12" s="2"/>
+      <c r="Y12" s="2"/>
+      <c r="Z12" s="2"/>
+    </row>
+    <row r="13" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>3</v>
       </c>
-      <c r="Z12" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA12" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC12" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
+      <c r="B13" s="1">
         <v>44169</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="2">
+      <c r="D13" s="2">
         <v>30.57</v>
       </c>
-      <c r="D13" s="2">
+      <c r="E13" s="2">
         <v>31.86</v>
       </c>
-      <c r="E13" s="2">
+      <c r="F13" s="2">
         <v>30.12</v>
       </c>
-      <c r="F13" s="2">
+      <c r="G13" s="2">
         <v>51</v>
-      </c>
-      <c r="G13" s="2">
-        <v>0</v>
       </c>
       <c r="H13" s="2">
         <v>19.28</v>
@@ -1799,49 +1595,32 @@
       <c r="V13" t="s">
         <v>2</v>
       </c>
-      <c r="W13" s="2">
-        <v>0</v>
-      </c>
-      <c r="X13" s="2">
-        <v>22.75</v>
-      </c>
-      <c r="Y13" t="s">
+      <c r="W13" s="2"/>
+      <c r="X13" s="2"/>
+      <c r="Y13" s="2"/>
+      <c r="Z13" s="2"/>
+    </row>
+    <row r="14" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>3</v>
       </c>
-      <c r="Z13" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA13" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB13" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC13" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
+      <c r="B14" s="1">
         <v>44169</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="2">
+      <c r="D14" s="2">
         <v>31.68</v>
       </c>
-      <c r="D14" s="2">
+      <c r="E14" s="2">
         <v>32.01</v>
       </c>
-      <c r="E14" s="2">
+      <c r="F14" s="2">
         <v>30.92</v>
       </c>
-      <c r="F14" s="2">
+      <c r="G14" s="2">
         <v>46.6</v>
-      </c>
-      <c r="G14" s="2">
-        <v>0</v>
       </c>
       <c r="H14" s="2">
         <v>18.84</v>
@@ -1888,49 +1667,32 @@
       <c r="V14" t="s">
         <v>2</v>
       </c>
-      <c r="W14" s="2">
-        <v>0</v>
-      </c>
-      <c r="X14" s="2">
-        <v>22.81</v>
-      </c>
-      <c r="Y14" t="s">
+      <c r="W14" s="2"/>
+      <c r="X14" s="2"/>
+      <c r="Y14" s="2"/>
+      <c r="Z14" s="2"/>
+    </row>
+    <row r="15" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>3</v>
       </c>
-      <c r="Z14" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA14" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB14" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC14" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
+      <c r="B15" s="1">
         <v>44169</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="2">
+      <c r="D15" s="2">
         <v>30.6</v>
       </c>
-      <c r="D15" s="2">
+      <c r="E15" s="2">
         <v>31.7</v>
       </c>
-      <c r="E15" s="2">
+      <c r="F15" s="2">
         <v>30.22</v>
       </c>
-      <c r="F15" s="2">
+      <c r="G15" s="2">
         <v>52.1</v>
-      </c>
-      <c r="G15" s="2">
-        <v>0</v>
       </c>
       <c r="H15" s="2">
         <v>19.649999999999999</v>
@@ -1977,49 +1739,32 @@
       <c r="V15" t="s">
         <v>2</v>
       </c>
-      <c r="W15" s="2">
-        <v>0</v>
-      </c>
-      <c r="X15" s="2">
-        <v>22.98</v>
-      </c>
-      <c r="Y15" t="s">
+      <c r="W15" s="2"/>
+      <c r="X15" s="2"/>
+      <c r="Y15" s="2"/>
+      <c r="Z15" s="2"/>
+    </row>
+    <row r="16" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>3</v>
       </c>
-      <c r="Z15" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA15" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB15" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC15" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
+      <c r="B16" s="1">
         <v>44169</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="2">
+      <c r="D16" s="2">
         <v>30.82</v>
       </c>
-      <c r="D16" s="2">
+      <c r="E16" s="2">
         <v>31.81</v>
       </c>
-      <c r="E16" s="2">
+      <c r="F16" s="2">
         <v>29.92</v>
       </c>
-      <c r="F16" s="2">
+      <c r="G16" s="2">
         <v>54.1</v>
-      </c>
-      <c r="G16" s="2">
-        <v>0</v>
       </c>
       <c r="H16" s="2">
         <v>20.46</v>
@@ -2066,49 +1811,32 @@
       <c r="V16" t="s">
         <v>2</v>
       </c>
-      <c r="W16" s="2">
-        <v>0</v>
-      </c>
-      <c r="X16" s="2">
-        <v>23.53</v>
-      </c>
-      <c r="Y16" t="s">
+      <c r="W16" s="2"/>
+      <c r="X16" s="2"/>
+      <c r="Y16" s="2"/>
+      <c r="Z16" s="2"/>
+    </row>
+    <row r="17" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>3</v>
       </c>
-      <c r="Z16" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA16" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB16" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC16" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
+      <c r="B17" s="1">
         <v>44169</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="2">
+      <c r="D17" s="2">
         <v>30.02</v>
       </c>
-      <c r="D17" s="2">
+      <c r="E17" s="2">
         <v>30.86</v>
       </c>
-      <c r="E17" s="2">
+      <c r="F17" s="2">
         <v>29.58</v>
       </c>
-      <c r="F17" s="2">
+      <c r="G17" s="2">
         <v>54.3</v>
-      </c>
-      <c r="G17" s="2">
-        <v>0</v>
       </c>
       <c r="H17" s="2">
         <v>19.78</v>
@@ -2155,49 +1883,32 @@
       <c r="V17" t="s">
         <v>2</v>
       </c>
-      <c r="W17" s="2">
-        <v>0</v>
-      </c>
-      <c r="X17" s="2">
-        <v>22.89</v>
-      </c>
-      <c r="Y17" t="s">
+      <c r="W17" s="2"/>
+      <c r="X17" s="2"/>
+      <c r="Y17" s="2"/>
+      <c r="Z17" s="2"/>
+    </row>
+    <row r="18" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>3</v>
       </c>
-      <c r="Z17" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA17" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB17" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC17" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
+      <c r="B18" s="1">
         <v>44169</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="2">
+      <c r="D18" s="2">
         <v>29.1</v>
       </c>
-      <c r="D18" s="2">
+      <c r="E18" s="2">
         <v>29.5</v>
       </c>
-      <c r="E18" s="2">
+      <c r="F18" s="2">
         <v>28.68</v>
       </c>
-      <c r="F18" s="2">
+      <c r="G18" s="2">
         <v>56.7</v>
-      </c>
-      <c r="G18" s="2">
-        <v>0</v>
       </c>
       <c r="H18" s="2">
         <v>19.62</v>
@@ -2244,49 +1955,32 @@
       <c r="V18" t="s">
         <v>2</v>
       </c>
-      <c r="W18" s="2">
-        <v>0</v>
-      </c>
-      <c r="X18" s="2">
-        <v>22.53</v>
-      </c>
-      <c r="Y18" t="s">
+      <c r="W18" s="2"/>
+      <c r="X18" s="2"/>
+      <c r="Y18" s="2"/>
+      <c r="Z18" s="2"/>
+    </row>
+    <row r="19" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>3</v>
       </c>
-      <c r="Z18" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA18" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB18" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC18" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
+      <c r="B19" s="1">
         <v>44169</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="2">
+      <c r="D19" s="2">
         <v>28.2</v>
       </c>
-      <c r="D19" s="2">
+      <c r="E19" s="2">
         <v>28.63</v>
       </c>
-      <c r="E19" s="2">
+      <c r="F19" s="2">
         <v>27.89</v>
       </c>
-      <c r="F19" s="2">
+      <c r="G19" s="2">
         <v>57.6</v>
-      </c>
-      <c r="G19" s="2">
-        <v>0</v>
       </c>
       <c r="H19" s="2">
         <v>19.04</v>
@@ -2333,49 +2027,32 @@
       <c r="V19" t="s">
         <v>2</v>
       </c>
-      <c r="W19" s="2">
-        <v>0</v>
-      </c>
-      <c r="X19" s="2">
-        <v>21.91</v>
-      </c>
-      <c r="Y19" t="s">
+      <c r="W19" s="2"/>
+      <c r="X19" s="2"/>
+      <c r="Y19" s="2"/>
+      <c r="Z19" s="2"/>
+    </row>
+    <row r="20" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>3</v>
       </c>
-      <c r="Z19" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA19" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB19" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC19" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
+      <c r="B20" s="1">
         <v>44169</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="2">
+      <c r="D20" s="2">
         <v>27.54</v>
       </c>
-      <c r="D20" s="2">
+      <c r="E20" s="2">
         <v>27.88</v>
       </c>
-      <c r="E20" s="2">
+      <c r="F20" s="2">
         <v>27.35</v>
       </c>
-      <c r="F20" s="2">
+      <c r="G20" s="2">
         <v>59.6</v>
-      </c>
-      <c r="G20" s="2">
-        <v>0</v>
       </c>
       <c r="H20" s="2">
         <v>18.97</v>
@@ -2422,49 +2099,32 @@
       <c r="V20" t="s">
         <v>2</v>
       </c>
-      <c r="W20" s="2">
-        <v>0</v>
-      </c>
-      <c r="X20" s="2">
-        <v>21.67</v>
-      </c>
-      <c r="Y20" t="s">
+      <c r="W20" s="2"/>
+      <c r="X20" s="2"/>
+      <c r="Y20" s="2"/>
+      <c r="Z20" s="2"/>
+    </row>
+    <row r="21" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>3</v>
       </c>
-      <c r="Z20" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA20" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB20" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC20" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
+      <c r="B21" s="1">
         <v>44169</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="2">
+      <c r="D21" s="2">
         <v>26.79</v>
       </c>
-      <c r="D21" s="2">
+      <c r="E21" s="2">
         <v>27.27</v>
       </c>
-      <c r="E21" s="2">
+      <c r="F21" s="2">
         <v>26.38</v>
       </c>
-      <c r="F21" s="2">
+      <c r="G21" s="2">
         <v>63.1</v>
-      </c>
-      <c r="G21" s="2">
-        <v>0</v>
       </c>
       <c r="H21" s="2">
         <v>19.18</v>
@@ -2511,49 +2171,32 @@
       <c r="V21" t="s">
         <v>2</v>
       </c>
-      <c r="W21" s="2">
-        <v>0</v>
-      </c>
-      <c r="X21" s="2">
-        <v>21.57</v>
-      </c>
-      <c r="Y21" t="s">
+      <c r="W21" s="2"/>
+      <c r="X21" s="2"/>
+      <c r="Y21" s="2"/>
+      <c r="Z21" s="2"/>
+    </row>
+    <row r="22" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>3</v>
       </c>
-      <c r="Z21" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA21" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB21" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC21" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
+      <c r="B22" s="1">
         <v>44169</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>27</v>
       </c>
-      <c r="C22" s="2">
+      <c r="D22" s="2">
         <v>25.95</v>
       </c>
-      <c r="D22" s="2">
+      <c r="E22" s="2">
         <v>26.31</v>
       </c>
-      <c r="E22" s="2">
+      <c r="F22" s="2">
         <v>25.7</v>
       </c>
-      <c r="F22" s="2">
+      <c r="G22" s="2">
         <v>63.6</v>
-      </c>
-      <c r="G22" s="2">
-        <v>0</v>
       </c>
       <c r="H22" s="2">
         <v>18.510000000000002</v>
@@ -2600,49 +2243,32 @@
       <c r="V22" t="s">
         <v>2</v>
       </c>
-      <c r="W22" s="2">
-        <v>0</v>
-      </c>
-      <c r="X22" s="2">
-        <v>20.9</v>
-      </c>
-      <c r="Y22" t="s">
+      <c r="W22" s="2"/>
+      <c r="X22" s="2"/>
+      <c r="Y22" s="2"/>
+      <c r="Z22" s="2"/>
+    </row>
+    <row r="23" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>3</v>
       </c>
-      <c r="Z22" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA22" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB22" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC22" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
+      <c r="B23" s="1">
         <v>44169</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>28</v>
       </c>
-      <c r="C23" s="2">
+      <c r="D23" s="2">
         <v>25.45</v>
       </c>
-      <c r="D23" s="2">
+      <c r="E23" s="2">
         <v>25.66</v>
       </c>
-      <c r="E23" s="2">
+      <c r="F23" s="2">
         <v>25.31</v>
       </c>
-      <c r="F23" s="2">
+      <c r="G23" s="2">
         <v>65.400000000000006</v>
-      </c>
-      <c r="G23" s="2">
-        <v>0</v>
       </c>
       <c r="H23" s="2">
         <v>18.489999999999998</v>
@@ -2689,49 +2315,32 @@
       <c r="V23" t="s">
         <v>2</v>
       </c>
-      <c r="W23" s="2">
-        <v>0</v>
-      </c>
-      <c r="X23" s="2">
-        <v>20.73</v>
-      </c>
-      <c r="Y23" t="s">
+      <c r="W23" s="2"/>
+      <c r="X23" s="2"/>
+      <c r="Y23" s="2"/>
+      <c r="Z23" s="2"/>
+    </row>
+    <row r="24" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>3</v>
       </c>
-      <c r="Z23" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA23" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB23" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC23" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
+      <c r="B24" s="1">
         <v>44169</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>29</v>
       </c>
-      <c r="C24" s="2">
+      <c r="D24" s="2">
         <v>25.08</v>
       </c>
-      <c r="D24" s="2">
+      <c r="E24" s="2">
         <v>25.29</v>
       </c>
-      <c r="E24" s="2">
+      <c r="F24" s="2">
         <v>24.94</v>
       </c>
-      <c r="F24" s="2">
+      <c r="G24" s="2">
         <v>67.2</v>
-      </c>
-      <c r="G24" s="2">
-        <v>0</v>
       </c>
       <c r="H24" s="2">
         <v>18.57</v>
@@ -2778,37 +2387,20 @@
       <c r="V24" t="s">
         <v>2</v>
       </c>
-      <c r="W24" s="2">
-        <v>0</v>
-      </c>
-      <c r="X24" s="2">
-        <v>20.67</v>
-      </c>
-      <c r="Y24" t="s">
+      <c r="W24" s="2"/>
+      <c r="X24" s="2"/>
+      <c r="Y24" s="2"/>
+      <c r="Z24" s="2"/>
+    </row>
+    <row r="25" spans="1:26" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>3</v>
       </c>
-      <c r="Z24" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA24" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB24" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC24" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:29" ht="10.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
+      <c r="B25" s="1">
         <v>44169</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>30</v>
-      </c>
-      <c r="C25" s="2">
-        <v>24.71</v>
       </c>
       <c r="D25" s="2">
         <v>24.71</v>
@@ -2817,10 +2409,10 @@
         <v>24.71</v>
       </c>
       <c r="F25" s="2">
+        <v>24.71</v>
+      </c>
+      <c r="G25" s="2">
         <v>70.099999999999994</v>
-      </c>
-      <c r="G25" s="2">
-        <v>0</v>
       </c>
       <c r="H25" s="2">
         <v>18.89</v>
@@ -2867,27 +2459,1690 @@
       <c r="V25" t="s">
         <v>2</v>
       </c>
-      <c r="W25" s="2">
-        <v>0</v>
-      </c>
-      <c r="X25" s="2">
-        <v>20.75</v>
-      </c>
-      <c r="Y25" t="s">
-        <v>3</v>
-      </c>
-      <c r="Z25" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA25" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB25" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC25" s="2">
-        <v>0</v>
-      </c>
+      <c r="W25" s="2"/>
+      <c r="X25" s="2"/>
+      <c r="Y25" s="2"/>
+      <c r="Z25" s="2"/>
+    </row>
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>62</v>
+      </c>
+      <c r="B26" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C26" t="s">
+        <v>60</v>
+      </c>
+      <c r="D26" s="2">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="E26" s="2">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="F26" s="2">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="G26" s="2">
+        <v>97</v>
+      </c>
+      <c r="H26" s="2">
+        <v>17.62</v>
+      </c>
+      <c r="I26" s="2">
+        <v>0</v>
+      </c>
+      <c r="J26" s="2">
+        <v>1.08</v>
+      </c>
+      <c r="K26" s="2">
+        <v>90</v>
+      </c>
+      <c r="L26" t="s">
+        <v>10</v>
+      </c>
+      <c r="M26" s="2">
+        <v>1.44</v>
+      </c>
+      <c r="N26" s="2">
+        <v>1.08</v>
+      </c>
+      <c r="O26" s="2">
+        <v>0</v>
+      </c>
+      <c r="P26" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="2">
+        <v>0</v>
+      </c>
+      <c r="R26" s="2">
+        <v>0</v>
+      </c>
+      <c r="S26" s="2">
+        <v>15.03</v>
+      </c>
+      <c r="T26" s="2">
+        <v>14.46</v>
+      </c>
+      <c r="U26" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V26" t="s">
+        <v>61</v>
+      </c>
+      <c r="W26" s="2"/>
+      <c r="X26" s="2"/>
+    </row>
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>62</v>
+      </c>
+      <c r="B27" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C27" t="s">
+        <v>63</v>
+      </c>
+      <c r="D27" s="2">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="E27" s="2">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="F27" s="2">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="G27" s="2">
+        <v>97</v>
+      </c>
+      <c r="H27" s="2">
+        <v>17.62</v>
+      </c>
+      <c r="I27" s="2">
+        <v>0</v>
+      </c>
+      <c r="J27" s="2">
+        <v>1.08</v>
+      </c>
+      <c r="K27" s="2">
+        <v>135</v>
+      </c>
+      <c r="L27" t="s">
+        <v>1</v>
+      </c>
+      <c r="M27" s="2">
+        <v>1.44</v>
+      </c>
+      <c r="N27" s="2">
+        <v>1.08</v>
+      </c>
+      <c r="O27" s="2">
+        <v>0</v>
+      </c>
+      <c r="P27" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="2">
+        <v>0</v>
+      </c>
+      <c r="R27" s="2">
+        <v>0</v>
+      </c>
+      <c r="S27" s="2">
+        <v>15.03</v>
+      </c>
+      <c r="T27" s="2">
+        <v>14.46</v>
+      </c>
+      <c r="U27" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V27" t="s">
+        <v>61</v>
+      </c>
+      <c r="W27" s="2"/>
+      <c r="X27" s="2"/>
+    </row>
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>62</v>
+      </c>
+      <c r="B28" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C28" t="s">
+        <v>64</v>
+      </c>
+      <c r="D28" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="E28" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="F28" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="G28" s="2">
+        <v>97</v>
+      </c>
+      <c r="H28" s="2">
+        <v>17.82</v>
+      </c>
+      <c r="I28" s="2">
+        <v>0</v>
+      </c>
+      <c r="J28" s="2">
+        <v>2.16</v>
+      </c>
+      <c r="K28" s="2">
+        <v>135</v>
+      </c>
+      <c r="L28" t="s">
+        <v>1</v>
+      </c>
+      <c r="M28" s="2">
+        <v>2.52</v>
+      </c>
+      <c r="N28" s="2">
+        <v>2.16</v>
+      </c>
+      <c r="O28" s="2">
+        <v>0</v>
+      </c>
+      <c r="P28" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="2">
+        <v>0</v>
+      </c>
+      <c r="R28" s="2">
+        <v>0</v>
+      </c>
+      <c r="S28" s="2">
+        <v>15.21</v>
+      </c>
+      <c r="T28" s="2">
+        <v>14.65</v>
+      </c>
+      <c r="U28" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V28" t="s">
+        <v>61</v>
+      </c>
+      <c r="W28" s="2"/>
+      <c r="X28" s="2"/>
+    </row>
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>62</v>
+      </c>
+      <c r="B29" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C29" t="s">
+        <v>65</v>
+      </c>
+      <c r="D29" s="2">
+        <v>18.7</v>
+      </c>
+      <c r="E29" s="2">
+        <v>18.7</v>
+      </c>
+      <c r="F29" s="2">
+        <v>18.7</v>
+      </c>
+      <c r="G29" s="2">
+        <v>97</v>
+      </c>
+      <c r="H29" s="2">
+        <v>18.21</v>
+      </c>
+      <c r="I29" s="2">
+        <v>0</v>
+      </c>
+      <c r="J29" s="2">
+        <v>2.88</v>
+      </c>
+      <c r="K29" s="2">
+        <v>113</v>
+      </c>
+      <c r="L29" t="s">
+        <v>66</v>
+      </c>
+      <c r="M29" s="2">
+        <v>3.96</v>
+      </c>
+      <c r="N29" s="2">
+        <v>2.88</v>
+      </c>
+      <c r="O29" s="2">
+        <v>0</v>
+      </c>
+      <c r="P29" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="2">
+        <v>0</v>
+      </c>
+      <c r="R29" s="2">
+        <v>0</v>
+      </c>
+      <c r="S29" s="2">
+        <v>15.58</v>
+      </c>
+      <c r="T29" s="2">
+        <v>15.02</v>
+      </c>
+      <c r="U29" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V29" t="s">
+        <v>61</v>
+      </c>
+      <c r="W29" s="2"/>
+      <c r="X29" s="2"/>
+    </row>
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>62</v>
+      </c>
+      <c r="B30" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C30" t="s">
+        <v>67</v>
+      </c>
+      <c r="D30" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="E30" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="F30" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="G30" s="2">
+        <v>96</v>
+      </c>
+      <c r="H30" s="2">
+        <v>18.149999999999999</v>
+      </c>
+      <c r="I30" s="2">
+        <v>0</v>
+      </c>
+      <c r="J30" s="2">
+        <v>2.88</v>
+      </c>
+      <c r="K30" s="2">
+        <v>113</v>
+      </c>
+      <c r="L30" t="s">
+        <v>66</v>
+      </c>
+      <c r="M30" s="2">
+        <v>3.96</v>
+      </c>
+      <c r="N30" s="2">
+        <v>2.88</v>
+      </c>
+      <c r="O30" s="2">
+        <v>0</v>
+      </c>
+      <c r="P30" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="2">
+        <v>0</v>
+      </c>
+      <c r="R30" s="2">
+        <v>0</v>
+      </c>
+      <c r="S30" s="2">
+        <v>15.52</v>
+      </c>
+      <c r="T30" s="2">
+        <v>14.96</v>
+      </c>
+      <c r="U30" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V30" t="s">
+        <v>61</v>
+      </c>
+      <c r="W30" s="2"/>
+      <c r="X30" s="2"/>
+    </row>
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>62</v>
+      </c>
+      <c r="B31" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C31" t="s">
+        <v>68</v>
+      </c>
+      <c r="D31" s="2">
+        <v>19</v>
+      </c>
+      <c r="E31" s="2">
+        <v>19</v>
+      </c>
+      <c r="F31" s="2">
+        <v>19</v>
+      </c>
+      <c r="G31" s="2">
+        <v>93</v>
+      </c>
+      <c r="H31" s="2">
+        <v>17.84</v>
+      </c>
+      <c r="I31" s="2">
+        <v>0</v>
+      </c>
+      <c r="J31" s="2">
+        <v>2.16</v>
+      </c>
+      <c r="K31" s="2">
+        <v>113</v>
+      </c>
+      <c r="L31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M31" s="2">
+        <v>2.52</v>
+      </c>
+      <c r="N31" s="2">
+        <v>2.16</v>
+      </c>
+      <c r="O31" s="2">
+        <v>0</v>
+      </c>
+      <c r="P31" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="2">
+        <v>1</v>
+      </c>
+      <c r="R31" s="2">
+        <v>0</v>
+      </c>
+      <c r="S31" s="2">
+        <v>15.23</v>
+      </c>
+      <c r="T31" s="2">
+        <v>14.68</v>
+      </c>
+      <c r="U31" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V31" t="s">
+        <v>61</v>
+      </c>
+      <c r="W31" s="2"/>
+      <c r="X31" s="2"/>
+    </row>
+    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>62</v>
+      </c>
+      <c r="B32" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C32" t="s">
+        <v>69</v>
+      </c>
+      <c r="D32" s="2">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="E32" s="2">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="F32" s="2">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="G32" s="2">
+        <v>90</v>
+      </c>
+      <c r="H32" s="2">
+        <v>17.91</v>
+      </c>
+      <c r="I32" s="2">
+        <v>0</v>
+      </c>
+      <c r="J32" s="2">
+        <v>2.16</v>
+      </c>
+      <c r="K32" s="2">
+        <v>90</v>
+      </c>
+      <c r="L32" t="s">
+        <v>10</v>
+      </c>
+      <c r="M32" s="2">
+        <v>2.52</v>
+      </c>
+      <c r="N32" s="2">
+        <v>2.16</v>
+      </c>
+      <c r="O32" s="2">
+        <v>0</v>
+      </c>
+      <c r="P32" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="2">
+        <v>1</v>
+      </c>
+      <c r="R32" s="2">
+        <v>0</v>
+      </c>
+      <c r="S32" s="2">
+        <v>15.3</v>
+      </c>
+      <c r="T32" s="2">
+        <v>14.76</v>
+      </c>
+      <c r="U32" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V32" t="s">
+        <v>61</v>
+      </c>
+      <c r="W32" s="2"/>
+      <c r="X32" s="2"/>
+    </row>
+    <row r="33" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>62</v>
+      </c>
+      <c r="B33" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C33" t="s">
+        <v>70</v>
+      </c>
+      <c r="D33" s="2">
+        <v>19.399999999999999</v>
+      </c>
+      <c r="E33" s="2">
+        <v>19.399999999999999</v>
+      </c>
+      <c r="F33" s="2">
+        <v>19.399999999999999</v>
+      </c>
+      <c r="G33" s="2">
+        <v>94</v>
+      </c>
+      <c r="H33" s="2">
+        <v>18.41</v>
+      </c>
+      <c r="I33" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J33" s="2">
+        <v>2.88</v>
+      </c>
+      <c r="K33" s="2">
+        <v>158</v>
+      </c>
+      <c r="L33" t="s">
+        <v>31</v>
+      </c>
+      <c r="M33" s="2">
+        <v>3.96</v>
+      </c>
+      <c r="N33" s="2">
+        <v>2.88</v>
+      </c>
+      <c r="O33" s="2">
+        <v>0</v>
+      </c>
+      <c r="P33" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="2">
+        <v>1</v>
+      </c>
+      <c r="R33" s="2">
+        <v>0</v>
+      </c>
+      <c r="S33" s="2">
+        <v>15.76</v>
+      </c>
+      <c r="T33" s="2">
+        <v>15.22</v>
+      </c>
+      <c r="U33" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V33" t="s">
+        <v>61</v>
+      </c>
+      <c r="W33" s="2"/>
+      <c r="X33" s="2"/>
+    </row>
+    <row r="34" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>62</v>
+      </c>
+      <c r="B34" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C34" t="s">
+        <v>71</v>
+      </c>
+      <c r="D34" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="E34" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="F34" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="G34" s="2">
+        <v>92</v>
+      </c>
+      <c r="H34" s="2">
+        <v>18.96</v>
+      </c>
+      <c r="I34" s="2">
+        <v>0</v>
+      </c>
+      <c r="J34" s="2">
+        <v>2.16</v>
+      </c>
+      <c r="K34" s="2">
+        <v>135</v>
+      </c>
+      <c r="L34" t="s">
+        <v>1</v>
+      </c>
+      <c r="M34" s="2">
+        <v>2.52</v>
+      </c>
+      <c r="N34" s="2">
+        <v>2.16</v>
+      </c>
+      <c r="O34" s="2">
+        <v>0</v>
+      </c>
+      <c r="P34" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="Q34" s="2">
+        <v>1</v>
+      </c>
+      <c r="R34" s="2">
+        <v>0.06</v>
+      </c>
+      <c r="S34" s="2">
+        <v>16.28</v>
+      </c>
+      <c r="T34" s="2">
+        <v>15.76</v>
+      </c>
+      <c r="U34" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V34" t="s">
+        <v>61</v>
+      </c>
+      <c r="W34" s="2"/>
+      <c r="X34" s="2"/>
+    </row>
+    <row r="35" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>62</v>
+      </c>
+      <c r="B35" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C35" t="s">
+        <v>72</v>
+      </c>
+      <c r="D35" s="2">
+        <v>26.2</v>
+      </c>
+      <c r="E35" s="2">
+        <v>26.2</v>
+      </c>
+      <c r="F35" s="2">
+        <v>26.2</v>
+      </c>
+      <c r="G35" s="2">
+        <v>65</v>
+      </c>
+      <c r="H35" s="2">
+        <v>19.100000000000001</v>
+      </c>
+      <c r="I35" s="2">
+        <v>0</v>
+      </c>
+      <c r="J35" s="2">
+        <v>2.88</v>
+      </c>
+      <c r="K35" s="2">
+        <v>45</v>
+      </c>
+      <c r="L35" t="s">
+        <v>12</v>
+      </c>
+      <c r="M35" s="2">
+        <v>3.96</v>
+      </c>
+      <c r="N35" s="2">
+        <v>2.88</v>
+      </c>
+      <c r="O35" s="2">
+        <v>0</v>
+      </c>
+      <c r="P35" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="Q35" s="2">
+        <v>1</v>
+      </c>
+      <c r="R35" s="2">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="S35" s="2">
+        <v>16.41</v>
+      </c>
+      <c r="T35" s="2">
+        <v>16.05</v>
+      </c>
+      <c r="U35" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V35" t="s">
+        <v>61</v>
+      </c>
+      <c r="W35" s="2"/>
+      <c r="X35" s="2"/>
+    </row>
+    <row r="36" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>62</v>
+      </c>
+      <c r="B36" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C36" t="s">
+        <v>73</v>
+      </c>
+      <c r="D36" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="E36" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="F36" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="G36" s="2">
+        <v>57</v>
+      </c>
+      <c r="H36" s="2">
+        <v>19.34</v>
+      </c>
+      <c r="I36" s="2">
+        <v>0</v>
+      </c>
+      <c r="J36" s="2">
+        <v>3.96</v>
+      </c>
+      <c r="K36" s="2">
+        <v>45</v>
+      </c>
+      <c r="L36" t="s">
+        <v>12</v>
+      </c>
+      <c r="M36" s="2">
+        <v>5.4</v>
+      </c>
+      <c r="N36" s="2">
+        <v>3.96</v>
+      </c>
+      <c r="O36" s="2">
+        <v>0</v>
+      </c>
+      <c r="P36" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q36" s="2">
+        <v>1</v>
+      </c>
+      <c r="R36" s="2">
+        <v>0.41</v>
+      </c>
+      <c r="S36" s="2">
+        <v>16.64</v>
+      </c>
+      <c r="T36" s="2">
+        <v>16.36</v>
+      </c>
+      <c r="U36" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V36" t="s">
+        <v>61</v>
+      </c>
+      <c r="W36" s="2"/>
+      <c r="X36" s="2"/>
+    </row>
+    <row r="37" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>62</v>
+      </c>
+      <c r="B37" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C37" t="s">
+        <v>74</v>
+      </c>
+      <c r="D37" s="2">
+        <v>31.1</v>
+      </c>
+      <c r="E37" s="2">
+        <v>31.1</v>
+      </c>
+      <c r="F37" s="2">
+        <v>31.1</v>
+      </c>
+      <c r="G37" s="2">
+        <v>52</v>
+      </c>
+      <c r="H37" s="2">
+        <v>20.079999999999998</v>
+      </c>
+      <c r="I37" s="2">
+        <v>0</v>
+      </c>
+      <c r="J37" s="2">
+        <v>3.96</v>
+      </c>
+      <c r="K37" s="2">
+        <v>45</v>
+      </c>
+      <c r="L37" t="s">
+        <v>12</v>
+      </c>
+      <c r="M37" s="2">
+        <v>5.4</v>
+      </c>
+      <c r="N37" s="2">
+        <v>3.96</v>
+      </c>
+      <c r="O37" s="2">
+        <v>0</v>
+      </c>
+      <c r="P37" s="2">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="Q37" s="2">
+        <v>1</v>
+      </c>
+      <c r="R37" s="2">
+        <v>0.49</v>
+      </c>
+      <c r="S37" s="2">
+        <v>17.38</v>
+      </c>
+      <c r="T37" s="2">
+        <v>17.21</v>
+      </c>
+      <c r="U37" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V37" t="s">
+        <v>61</v>
+      </c>
+      <c r="W37" s="2"/>
+      <c r="X37" s="2"/>
+    </row>
+    <row r="38" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C38" t="s">
+        <v>75</v>
+      </c>
+      <c r="D38" s="2">
+        <v>31.1</v>
+      </c>
+      <c r="E38" s="2">
+        <v>31.1</v>
+      </c>
+      <c r="F38" s="2">
+        <v>31.1</v>
+      </c>
+      <c r="G38" s="2">
+        <v>52</v>
+      </c>
+      <c r="H38" s="2">
+        <v>20.079999999999998</v>
+      </c>
+      <c r="I38" s="2">
+        <v>0</v>
+      </c>
+      <c r="J38" s="2">
+        <v>6.84</v>
+      </c>
+      <c r="K38" s="2">
+        <v>68</v>
+      </c>
+      <c r="L38" t="s">
+        <v>19</v>
+      </c>
+      <c r="M38" s="2">
+        <v>9.36</v>
+      </c>
+      <c r="N38" s="2">
+        <v>6.84</v>
+      </c>
+      <c r="O38" s="2">
+        <v>0</v>
+      </c>
+      <c r="P38" s="2">
+        <v>2.5</v>
+      </c>
+      <c r="Q38" s="2">
+        <v>1</v>
+      </c>
+      <c r="R38" s="2">
+        <v>0.54</v>
+      </c>
+      <c r="S38" s="2">
+        <v>17.38</v>
+      </c>
+      <c r="T38" s="2">
+        <v>17.21</v>
+      </c>
+      <c r="U38" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V38" t="s">
+        <v>61</v>
+      </c>
+      <c r="W38" s="2"/>
+      <c r="X38" s="2"/>
+    </row>
+    <row r="39" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>62</v>
+      </c>
+      <c r="B39" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C39" t="s">
+        <v>76</v>
+      </c>
+      <c r="D39" s="2">
+        <v>30.1</v>
+      </c>
+      <c r="E39" s="2">
+        <v>30.1</v>
+      </c>
+      <c r="F39" s="2">
+        <v>30.1</v>
+      </c>
+      <c r="G39" s="2">
+        <v>53</v>
+      </c>
+      <c r="H39" s="2">
+        <v>19.46</v>
+      </c>
+      <c r="I39" s="2">
+        <v>0</v>
+      </c>
+      <c r="J39" s="2">
+        <v>6.12</v>
+      </c>
+      <c r="K39" s="2">
+        <v>90</v>
+      </c>
+      <c r="L39" t="s">
+        <v>10</v>
+      </c>
+      <c r="M39" s="2">
+        <v>7.92</v>
+      </c>
+      <c r="N39" s="2">
+        <v>6.12</v>
+      </c>
+      <c r="O39" s="2">
+        <v>0</v>
+      </c>
+      <c r="P39" s="2">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="Q39" s="2">
+        <v>1</v>
+      </c>
+      <c r="R39" s="2">
+        <v>0.49</v>
+      </c>
+      <c r="S39" s="2">
+        <v>16.77</v>
+      </c>
+      <c r="T39" s="2">
+        <v>16.54</v>
+      </c>
+      <c r="U39" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V39" t="s">
+        <v>61</v>
+      </c>
+      <c r="W39" s="2"/>
+      <c r="X39" s="2"/>
+    </row>
+    <row r="40" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C40" t="s">
+        <v>77</v>
+      </c>
+      <c r="D40" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="E40" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="F40" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="G40" s="2">
+        <v>59</v>
+      </c>
+      <c r="H40" s="2">
+        <v>19.89</v>
+      </c>
+      <c r="I40" s="2">
+        <v>0</v>
+      </c>
+      <c r="J40" s="2">
+        <v>9</v>
+      </c>
+      <c r="K40" s="2">
+        <v>90</v>
+      </c>
+      <c r="L40" t="s">
+        <v>10</v>
+      </c>
+      <c r="M40" s="2">
+        <v>11.88</v>
+      </c>
+      <c r="N40" s="2">
+        <v>9</v>
+      </c>
+      <c r="O40" s="2">
+        <v>0</v>
+      </c>
+      <c r="P40" s="2">
+        <v>1.3</v>
+      </c>
+      <c r="Q40" s="2">
+        <v>1</v>
+      </c>
+      <c r="R40" s="2">
+        <v>0.31</v>
+      </c>
+      <c r="S40" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="T40" s="2">
+        <v>16.93</v>
+      </c>
+      <c r="U40" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V40" t="s">
+        <v>61</v>
+      </c>
+      <c r="W40" s="2"/>
+      <c r="X40" s="2"/>
+    </row>
+    <row r="41" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>62</v>
+      </c>
+      <c r="B41" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C41" t="s">
+        <v>78</v>
+      </c>
+      <c r="D41" s="2">
+        <v>28.1</v>
+      </c>
+      <c r="E41" s="2">
+        <v>28.1</v>
+      </c>
+      <c r="F41" s="2">
+        <v>28.1</v>
+      </c>
+      <c r="G41" s="2">
+        <v>63</v>
+      </c>
+      <c r="H41" s="2">
+        <v>20.39</v>
+      </c>
+      <c r="I41" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J41" s="2">
+        <v>6.12</v>
+      </c>
+      <c r="K41" s="2">
+        <v>68</v>
+      </c>
+      <c r="L41" t="s">
+        <v>19</v>
+      </c>
+      <c r="M41" s="2">
+        <v>7.92</v>
+      </c>
+      <c r="N41" s="2">
+        <v>6.12</v>
+      </c>
+      <c r="O41" s="2">
+        <v>0</v>
+      </c>
+      <c r="P41" s="2">
+        <v>1.2</v>
+      </c>
+      <c r="Q41" s="2">
+        <v>1</v>
+      </c>
+      <c r="R41" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="S41" s="2">
+        <v>17.71</v>
+      </c>
+      <c r="T41" s="2">
+        <v>17.440000000000001</v>
+      </c>
+      <c r="U41" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V41" t="s">
+        <v>61</v>
+      </c>
+      <c r="W41" s="2"/>
+      <c r="X41" s="2"/>
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>62</v>
+      </c>
+      <c r="B42" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C42" t="s">
+        <v>79</v>
+      </c>
+      <c r="D42" s="2">
+        <v>29.2</v>
+      </c>
+      <c r="E42" s="2">
+        <v>29.2</v>
+      </c>
+      <c r="F42" s="2">
+        <v>29.2</v>
+      </c>
+      <c r="G42" s="2">
+        <v>61</v>
+      </c>
+      <c r="H42" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="I42" s="2">
+        <v>0</v>
+      </c>
+      <c r="J42" s="2">
+        <v>9</v>
+      </c>
+      <c r="K42" s="2">
+        <v>90</v>
+      </c>
+      <c r="L42" t="s">
+        <v>10</v>
+      </c>
+      <c r="M42" s="2">
+        <v>11.88</v>
+      </c>
+      <c r="N42" s="2">
+        <v>9</v>
+      </c>
+      <c r="O42" s="2">
+        <v>0</v>
+      </c>
+      <c r="P42" s="2">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="Q42" s="2">
+        <v>1</v>
+      </c>
+      <c r="R42" s="2">
+        <v>0.45</v>
+      </c>
+      <c r="S42" s="2">
+        <v>18.239999999999998</v>
+      </c>
+      <c r="T42" s="2">
+        <v>18.04</v>
+      </c>
+      <c r="U42" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V42" t="s">
+        <v>61</v>
+      </c>
+      <c r="W42" s="2"/>
+      <c r="X42" s="2"/>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>62</v>
+      </c>
+      <c r="B43" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C43" t="s">
+        <v>80</v>
+      </c>
+      <c r="D43" s="2">
+        <v>26</v>
+      </c>
+      <c r="E43" s="2">
+        <v>26</v>
+      </c>
+      <c r="F43" s="2">
+        <v>26</v>
+      </c>
+      <c r="G43" s="2">
+        <v>71</v>
+      </c>
+      <c r="H43" s="2">
+        <v>20.329999999999998</v>
+      </c>
+      <c r="I43" s="2">
+        <v>0</v>
+      </c>
+      <c r="J43" s="2">
+        <v>5.04</v>
+      </c>
+      <c r="K43" s="2">
+        <v>68</v>
+      </c>
+      <c r="L43" t="s">
+        <v>19</v>
+      </c>
+      <c r="M43" s="2">
+        <v>6.84</v>
+      </c>
+      <c r="N43" s="2">
+        <v>5.04</v>
+      </c>
+      <c r="O43" s="2">
+        <v>0</v>
+      </c>
+      <c r="P43" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="Q43" s="2">
+        <v>1</v>
+      </c>
+      <c r="R43" s="2">
+        <v>0.16</v>
+      </c>
+      <c r="S43" s="2">
+        <v>17.64</v>
+      </c>
+      <c r="T43" s="2">
+        <v>17.309999999999999</v>
+      </c>
+      <c r="U43" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V43" t="s">
+        <v>61</v>
+      </c>
+      <c r="W43" s="2"/>
+      <c r="X43" s="2"/>
+    </row>
+    <row r="44" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>62</v>
+      </c>
+      <c r="B44" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C44" t="s">
+        <v>81</v>
+      </c>
+      <c r="D44" s="2">
+        <v>24.4</v>
+      </c>
+      <c r="E44" s="2">
+        <v>24.4</v>
+      </c>
+      <c r="F44" s="2">
+        <v>24.4</v>
+      </c>
+      <c r="G44" s="2">
+        <v>79</v>
+      </c>
+      <c r="H44" s="2">
+        <v>20.52</v>
+      </c>
+      <c r="I44" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="J44" s="2">
+        <v>5.04</v>
+      </c>
+      <c r="K44" s="2">
+        <v>113</v>
+      </c>
+      <c r="L44" t="s">
+        <v>66</v>
+      </c>
+      <c r="M44" s="2">
+        <v>6.84</v>
+      </c>
+      <c r="N44" s="2">
+        <v>5.04</v>
+      </c>
+      <c r="O44" s="2">
+        <v>100</v>
+      </c>
+      <c r="P44" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="Q44" s="2">
+        <v>0</v>
+      </c>
+      <c r="R44" s="2">
+        <v>0.11</v>
+      </c>
+      <c r="S44" s="2">
+        <v>17.84</v>
+      </c>
+      <c r="T44" s="2">
+        <v>17.46</v>
+      </c>
+      <c r="U44" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V44" t="s">
+        <v>61</v>
+      </c>
+      <c r="W44" s="2"/>
+      <c r="X44" s="2"/>
+    </row>
+    <row r="45" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>62</v>
+      </c>
+      <c r="B45" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C45" t="s">
+        <v>82</v>
+      </c>
+      <c r="D45" s="2">
+        <v>22.9</v>
+      </c>
+      <c r="E45" s="2">
+        <v>22.9</v>
+      </c>
+      <c r="F45" s="2">
+        <v>22.9</v>
+      </c>
+      <c r="G45" s="2">
+        <v>87</v>
+      </c>
+      <c r="H45" s="2">
+        <v>20.62</v>
+      </c>
+      <c r="I45" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="J45" s="2">
+        <v>3.96</v>
+      </c>
+      <c r="K45" s="2">
+        <v>90</v>
+      </c>
+      <c r="L45" t="s">
+        <v>10</v>
+      </c>
+      <c r="M45" s="2">
+        <v>5.4</v>
+      </c>
+      <c r="N45" s="2">
+        <v>3.96</v>
+      </c>
+      <c r="O45" s="2">
+        <v>100</v>
+      </c>
+      <c r="P45" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="Q45" s="2">
+        <v>0</v>
+      </c>
+      <c r="R45" s="2">
+        <v>0.08</v>
+      </c>
+      <c r="S45" s="2">
+        <v>17.940000000000001</v>
+      </c>
+      <c r="T45" s="2">
+        <v>17.53</v>
+      </c>
+      <c r="U45" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V45" t="s">
+        <v>61</v>
+      </c>
+      <c r="W45" s="2"/>
+      <c r="X45" s="2"/>
+    </row>
+    <row r="46" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>62</v>
+      </c>
+      <c r="B46" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C46" t="s">
+        <v>83</v>
+      </c>
+      <c r="D46" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E46" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="F46" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="G46" s="2">
+        <v>91</v>
+      </c>
+      <c r="H46" s="2">
+        <v>20.56</v>
+      </c>
+      <c r="I46" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J46" s="2">
+        <v>5.04</v>
+      </c>
+      <c r="K46" s="2">
+        <v>135</v>
+      </c>
+      <c r="L46" t="s">
+        <v>1</v>
+      </c>
+      <c r="M46" s="2">
+        <v>6.84</v>
+      </c>
+      <c r="N46" s="2">
+        <v>5.04</v>
+      </c>
+      <c r="O46" s="2">
+        <v>100</v>
+      </c>
+      <c r="P46" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="2">
+        <v>0</v>
+      </c>
+      <c r="R46" s="2">
+        <v>0</v>
+      </c>
+      <c r="S46" s="2">
+        <v>17.88</v>
+      </c>
+      <c r="T46" s="2">
+        <v>17.440000000000001</v>
+      </c>
+      <c r="U46" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V46" t="s">
+        <v>61</v>
+      </c>
+      <c r="W46" s="2"/>
+      <c r="X46" s="2"/>
+    </row>
+    <row r="47" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>62</v>
+      </c>
+      <c r="B47" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C47" t="s">
+        <v>84</v>
+      </c>
+      <c r="D47" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="E47" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="F47" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="G47" s="2">
+        <v>94</v>
+      </c>
+      <c r="H47" s="2">
+        <v>19.899999999999999</v>
+      </c>
+      <c r="I47" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="J47" s="2">
+        <v>5.04</v>
+      </c>
+      <c r="K47" s="2">
+        <v>113</v>
+      </c>
+      <c r="L47" t="s">
+        <v>66</v>
+      </c>
+      <c r="M47" s="2">
+        <v>6.84</v>
+      </c>
+      <c r="N47" s="2">
+        <v>5.04</v>
+      </c>
+      <c r="O47" s="2">
+        <v>100</v>
+      </c>
+      <c r="P47" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q47" s="2">
+        <v>0</v>
+      </c>
+      <c r="R47" s="2">
+        <v>0</v>
+      </c>
+      <c r="S47" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="T47" s="2">
+        <v>16.71</v>
+      </c>
+      <c r="U47" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V47" t="s">
+        <v>61</v>
+      </c>
+      <c r="W47" s="2"/>
+      <c r="X47" s="2"/>
+    </row>
+    <row r="48" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>62</v>
+      </c>
+      <c r="B48" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C48" t="s">
+        <v>85</v>
+      </c>
+      <c r="D48" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="E48" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="F48" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="G48" s="2">
+        <v>95</v>
+      </c>
+      <c r="H48" s="2">
+        <v>19.47</v>
+      </c>
+      <c r="I48" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J48" s="2">
+        <v>5.04</v>
+      </c>
+      <c r="K48" s="2">
+        <v>135</v>
+      </c>
+      <c r="L48" t="s">
+        <v>1</v>
+      </c>
+      <c r="M48" s="2">
+        <v>6.84</v>
+      </c>
+      <c r="N48" s="2">
+        <v>5.04</v>
+      </c>
+      <c r="O48" s="2">
+        <v>100</v>
+      </c>
+      <c r="P48" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q48" s="2">
+        <v>0</v>
+      </c>
+      <c r="R48" s="2">
+        <v>0</v>
+      </c>
+      <c r="S48" s="2">
+        <v>16.78</v>
+      </c>
+      <c r="T48" s="2">
+        <v>16.27</v>
+      </c>
+      <c r="U48" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V48" t="s">
+        <v>61</v>
+      </c>
+      <c r="W48" s="2"/>
+      <c r="X48" s="2"/>
+    </row>
+    <row r="49" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>62</v>
+      </c>
+      <c r="B49" s="1">
+        <v>43853</v>
+      </c>
+      <c r="C49" t="s">
+        <v>86</v>
+      </c>
+      <c r="D49" s="2">
+        <v>19.899999999999999</v>
+      </c>
+      <c r="E49" s="2">
+        <v>19.899999999999999</v>
+      </c>
+      <c r="F49" s="2">
+        <v>19.899999999999999</v>
+      </c>
+      <c r="G49" s="2">
+        <v>97</v>
+      </c>
+      <c r="H49" s="2">
+        <v>19.41</v>
+      </c>
+      <c r="I49" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J49" s="2">
+        <v>3.96</v>
+      </c>
+      <c r="K49" s="2">
+        <v>135</v>
+      </c>
+      <c r="L49" t="s">
+        <v>1</v>
+      </c>
+      <c r="M49" s="2">
+        <v>5.4</v>
+      </c>
+      <c r="N49" s="2">
+        <v>3.96</v>
+      </c>
+      <c r="O49" s="2">
+        <v>100</v>
+      </c>
+      <c r="P49" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q49" s="2">
+        <v>0</v>
+      </c>
+      <c r="R49" s="2">
+        <v>0</v>
+      </c>
+      <c r="S49" s="2">
+        <v>16.72</v>
+      </c>
+      <c r="T49" s="2">
+        <v>16.2</v>
+      </c>
+      <c r="U49" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="V49" t="s">
+        <v>61</v>
+      </c>
+      <c r="W49" s="2"/>
+      <c r="X49" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>